<commit_message>
Formula & SQL guide with practice links, resizable split + full screen, GridCraft web build, wider xlsx columns
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TLEvBfKCpDrK43nEFcLg7p
</commit_message>
<xml_diff>
--- a/public/data/xlsx/etl1.xlsx
+++ b/public/data/xlsx/etl1.xlsx
@@ -420,6 +420,17 @@
   </sheetPr>
   <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">

</xml_diff>